<commit_message>
Annuaire des notaires : note de livraison — décisions du 18 oct. (suite) et libellés corrigés
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/livraison-notaires-confirmation/Libelles-en-ht-a-valider-2026-10-18.xlsx
+++ b/docs/livraison-notaires-confirmation/Libelles-en-ht-a-valider-2026-10-18.xlsx
@@ -557,12 +557,12 @@
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>Carte judiciaire et notaires</t>
+          <t>Carte judiciaire et des notaires</t>
         </is>
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t>Judicial map and notaries</t>
+          <t>Judicial map and of notaries</t>
         </is>
       </c>
       <c r="F6" s="5" t="inlineStr">
@@ -570,9 +570,17 @@
           <t>Kat jidisyè ak notè yo</t>
         </is>
       </c>
-      <c r="G6" s="6" t="inlineStr"/>
-      <c r="H6" s="6" t="inlineStr"/>
-      <c r="I6" s="6" t="inlineStr"/>
+      <c r="G6" s="6" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="H6" s="6" t="n"/>
+      <c r="I6" s="6" t="inlineStr">
+        <is>
+          <t>Corrigé par Me Vaval le 18 oct. (FR, EN) — appliqué</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="5" t="n">
@@ -1854,12 +1862,20 @@
       </c>
       <c r="F45" s="5" t="inlineStr">
         <is>
-          <t>Adrès etid la pa ranseye</t>
-        </is>
-      </c>
-      <c r="G45" s="6" t="inlineStr"/>
-      <c r="H45" s="6" t="inlineStr"/>
-      <c r="I45" s="6" t="inlineStr"/>
+          <t>Adrès etid la pa kominike</t>
+        </is>
+      </c>
+      <c r="G45" s="6" t="n"/>
+      <c r="H45" s="6" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="I45" s="6" t="inlineStr">
+        <is>
+          <t>Créole corrigé par Me Vaval le 18 oct. — appliqué</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="5" t="n">
@@ -2448,12 +2464,20 @@
       </c>
       <c r="F63" s="5" t="inlineStr">
         <is>
-          <t>Enfòmasyon notè a konfime.</t>
-        </is>
-      </c>
-      <c r="G63" s="6" t="inlineStr"/>
-      <c r="H63" s="6" t="inlineStr"/>
-      <c r="I63" s="6" t="inlineStr"/>
+          <t>Notè a konfime enfòmasyon an.</t>
+        </is>
+      </c>
+      <c r="G63" s="6" t="n"/>
+      <c r="H63" s="6" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="I63" s="6" t="inlineStr">
+        <is>
+          <t>Créole corrigé par Me Vaval le 18 oct. — appliqué</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="5" t="n">
@@ -2481,12 +2505,16 @@
       </c>
       <c r="F64" s="5" t="inlineStr">
         <is>
-          <t>Enfòmasyon notè a konfime</t>
+          <t>Notè a konfime enfòmasyon an</t>
         </is>
       </c>
       <c r="G64" s="6" t="inlineStr"/>
       <c r="H64" s="6" t="inlineStr"/>
-      <c r="I64" s="6" t="inlineStr"/>
+      <c r="I64" s="6" t="inlineStr">
+        <is>
+          <t>Aligné sur sa correction de l’infobulle — à valider</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="5" t="n">
@@ -2570,22 +2598,26 @@
       </c>
       <c r="D67" s="5" t="inlineStr">
         <is>
-          <t>Proposez une correction ou confirmez les informations affichées. La demande est examinée par le Master Admin : rien n’est publié avant vérification.</t>
+          <t>Proposez une correction ou confirmez les informations affichées. La demande est examinée par l’Administrateur : rien n’est publié avant vérification.</t>
         </is>
       </c>
       <c r="E67" s="5" t="inlineStr">
         <is>
-          <t>Suggest a correction or confirm the information shown. The request is reviewed by the Master Admin: nothing is published before it is checked.</t>
+          <t>Suggest a correction or confirm the information shown. The request is reviewed by the Administrator: nothing is published before it is checked.</t>
         </is>
       </c>
       <c r="F67" s="5" t="inlineStr">
         <is>
-          <t>Pwopoze yon koreksyon oswa konfime enfòmasyon ki afiche yo. Master Admin nan ap egzamine demann lan : anyen p ap pibliye anvan verifikasyon.</t>
+          <t>Pwopoze yon koreksyon oswa konfime enfòmasyon ki afiche yo. Administratè a ap egzamine demann lan : anyen p ap pibliye anvan verifikasyon.</t>
         </is>
       </c>
       <c r="G67" s="6" t="inlineStr"/>
       <c r="H67" s="6" t="inlineStr"/>
-      <c r="I67" s="6" t="inlineStr"/>
+      <c r="I67" s="6" t="inlineStr">
+        <is>
+          <t>Aligné sur « l’Administrateur » (sa correction du message d’envoi) — à valider</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="5" t="n">
@@ -2636,22 +2668,34 @@
       </c>
       <c r="D69" s="5" t="inlineStr">
         <is>
-          <t>Votre demande a été transmise au Master Admin pour examen.</t>
+          <t>Votre demande a été transmise à l’Administrateur pour examen.</t>
         </is>
       </c>
       <c r="E69" s="5" t="inlineStr">
         <is>
-          <t>Your request has been sent to the Master Admin for review.</t>
+          <t>Your request has been sent to the Administrator for review.</t>
         </is>
       </c>
       <c r="F69" s="5" t="inlineStr">
         <is>
-          <t>Demann ou an voye bay Master Admin nan pou egzamen.</t>
-        </is>
-      </c>
-      <c r="G69" s="6" t="inlineStr"/>
-      <c r="H69" s="6" t="inlineStr"/>
-      <c r="I69" s="6" t="inlineStr"/>
+          <t>Demann ou a voye bay Administratè a pou egzamen.</t>
+        </is>
+      </c>
+      <c r="G69" s="6" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="H69" s="6" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="I69" s="6" t="inlineStr">
+        <is>
+          <t>Corrigé par Me Vaval le 18 oct. (FR, EN, HT) — appliqué</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="5" t="n">
@@ -2877,12 +2921,16 @@
       </c>
       <c r="F76" s="5" t="inlineStr">
         <is>
-          <t>pa ranseye</t>
+          <t>pa kominike</t>
         </is>
       </c>
       <c r="G76" s="6" t="inlineStr"/>
       <c r="H76" s="6" t="inlineStr"/>
-      <c r="I76" s="6" t="inlineStr"/>
+      <c r="I76" s="6" t="inlineStr">
+        <is>
+          <t>Aligné sur « pa kominike » — à valider</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="5" t="n">

</xml_diff>

<commit_message>
Carte judiciaire : titre anglais « Map of courts and notaries » ; libellés en/ht validés par Me Vaval
« leave it as you prefer » (titre) et « auto confirm » (les 67 libellés restants), 18 oct. 2026.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/livraison-notaires-confirmation/Libelles-en-ht-a-valider-2026-10-18.xlsx
+++ b/docs/livraison-notaires-confirmation/Libelles-en-ht-a-valider-2026-10-18.xlsx
@@ -476,7 +476,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Carte judiciaire et notaires — libellés anglais et créoles à valider (18 oct. 2026)</t>
+          <t>Carte judiciaire et notaires — libellés anglais et créoles (VALIDÉS le 18 oct. 2026)</t>
         </is>
       </c>
     </row>
@@ -562,7 +562,7 @@
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t>Judicial map and of notaries</t>
+          <t>Map of courts and notaries</t>
         </is>
       </c>
       <c r="F6" s="5" t="inlineStr">
@@ -575,10 +575,14 @@
           <t>Oui</t>
         </is>
       </c>
-      <c r="H6" s="6" t="n"/>
+      <c r="H6" s="6" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
       <c r="I6" s="6" t="inlineStr">
         <is>
-          <t>Corrigé par Me Vaval le 18 oct. (FR, EN) — appliqué</t>
+          <t>FR corrigé par Me Vaval ; EN : « Map of courts and notaries » (« leave it as you prefer ») ; HT confirmé</t>
         </is>
       </c>
     </row>
@@ -611,9 +615,21 @@
           <t>Jwenn yon jiridiksyon oswa yon notè, toupatou ann Ayiti.</t>
         </is>
       </c>
-      <c r="G7" s="6" t="inlineStr"/>
-      <c r="H7" s="6" t="inlineStr"/>
-      <c r="I7" s="6" t="inlineStr"/>
+      <c r="G7" s="6" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="H7" s="6" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="I7" s="6" t="inlineStr">
+        <is>
+          <t>Confirmé par Me Vaval le 18 oct. (« auto confirm »)</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="5" t="n">
@@ -644,9 +660,21 @@
           <t>Vi kat jidisyè a</t>
         </is>
       </c>
-      <c r="G8" s="6" t="inlineStr"/>
-      <c r="H8" s="6" t="inlineStr"/>
-      <c r="I8" s="6" t="inlineStr"/>
+      <c r="G8" s="6" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="H8" s="6" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="I8" s="6" t="inlineStr">
+        <is>
+          <t>Confirmé par Me Vaval le 18 oct. (« auto confirm »)</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="5" t="n">
@@ -677,9 +705,21 @@
           <t>Jiridiksyon yo</t>
         </is>
       </c>
-      <c r="G9" s="6" t="inlineStr"/>
-      <c r="H9" s="6" t="inlineStr"/>
-      <c r="I9" s="6" t="inlineStr"/>
+      <c r="G9" s="6" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="H9" s="6" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="I9" s="6" t="inlineStr">
+        <is>
+          <t>Confirmé par Me Vaval le 18 oct. (« auto confirm »)</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="5" t="n">
@@ -710,9 +750,21 @@
           <t>Notè yo</t>
         </is>
       </c>
-      <c r="G10" s="6" t="inlineStr"/>
-      <c r="H10" s="6" t="inlineStr"/>
-      <c r="I10" s="6" t="inlineStr"/>
+      <c r="G10" s="6" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="H10" s="6" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="I10" s="6" t="inlineStr">
+        <is>
+          <t>Confirmé par Me Vaval le 18 oct. (« auto confirm »)</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="5" t="n">
@@ -743,9 +795,21 @@
           <t>Gade anyè notè yo</t>
         </is>
       </c>
-      <c r="G11" s="6" t="inlineStr"/>
-      <c r="H11" s="6" t="inlineStr"/>
-      <c r="I11" s="6" t="inlineStr"/>
+      <c r="G11" s="6" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="H11" s="6" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="I11" s="6" t="inlineStr">
+        <is>
+          <t>Confirmé par Me Vaval le 18 oct. (« auto confirm »)</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="5" t="n">
@@ -776,9 +840,21 @@
           <t>Anyè notè Ayiti yo — kat jidisyè | Agora</t>
         </is>
       </c>
-      <c r="G12" s="6" t="inlineStr"/>
-      <c r="H12" s="6" t="inlineStr"/>
-      <c r="I12" s="6" t="inlineStr"/>
+      <c r="G12" s="6" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="H12" s="6" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="I12" s="6" t="inlineStr">
+        <is>
+          <t>Confirmé par Me Vaval le 18 oct. (« auto confirm »)</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="5" t="n">
@@ -809,9 +885,21 @@
           <t>Anyè notè Ayiti yo, dapre lis Ministè Lajistis la, klase pa jiridiksyon, ak kat komin komisyon yo.</t>
         </is>
       </c>
-      <c r="G13" s="6" t="inlineStr"/>
-      <c r="H13" s="6" t="inlineStr"/>
-      <c r="I13" s="6" t="inlineStr"/>
+      <c r="G13" s="6" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="H13" s="6" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="I13" s="6" t="inlineStr">
+        <is>
+          <t>Confirmé par Me Vaval le 18 oct. (« auto confirm »)</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="5" t="n">
@@ -842,9 +930,21 @@
           <t>Kowòdone etid notè yo</t>
         </is>
       </c>
-      <c r="G14" s="6" t="inlineStr"/>
-      <c r="H14" s="6" t="inlineStr"/>
-      <c r="I14" s="6" t="inlineStr"/>
+      <c r="G14" s="6" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="H14" s="6" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="I14" s="6" t="inlineStr">
+        <is>
+          <t>Confirmé par Me Vaval le 18 oct. (« auto confirm »)</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="5" t="n">
@@ -875,9 +975,21 @@
           <t>Anyè notè yo</t>
         </is>
       </c>
-      <c r="G15" s="6" t="inlineStr"/>
-      <c r="H15" s="6" t="inlineStr"/>
-      <c r="I15" s="6" t="inlineStr"/>
+      <c r="G15" s="6" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="H15" s="6" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="I15" s="6" t="inlineStr">
+        <is>
+          <t>Confirmé par Me Vaval le 18 oct. (« auto confirm »)</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="5" t="n">
@@ -908,9 +1020,21 @@
           <t>Chèche yon notè oswa yon komin</t>
         </is>
       </c>
-      <c r="G16" s="6" t="inlineStr"/>
-      <c r="H16" s="6" t="inlineStr"/>
-      <c r="I16" s="6" t="inlineStr"/>
+      <c r="G16" s="6" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="H16" s="6" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="I16" s="6" t="inlineStr">
+        <is>
+          <t>Confirmé par Me Vaval le 18 oct. (« auto confirm »)</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="5" t="n">
@@ -941,9 +1065,21 @@
           <t>Chèche yon notè oswa yon komin…</t>
         </is>
       </c>
-      <c r="G17" s="6" t="inlineStr"/>
-      <c r="H17" s="6" t="inlineStr"/>
-      <c r="I17" s="6" t="inlineStr"/>
+      <c r="G17" s="6" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="H17" s="6" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="I17" s="6" t="inlineStr">
+        <is>
+          <t>Confirmé par Me Vaval le 18 oct. (« auto confirm »)</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="5" t="n">
@@ -974,9 +1110,21 @@
           <t>Chèche</t>
         </is>
       </c>
-      <c r="G18" s="6" t="inlineStr"/>
-      <c r="H18" s="6" t="inlineStr"/>
-      <c r="I18" s="6" t="inlineStr"/>
+      <c r="G18" s="6" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="H18" s="6" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="I18" s="6" t="inlineStr">
+        <is>
+          <t>Confirmé par Me Vaval le 18 oct. (« auto confirm »)</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="5" t="n">
@@ -1007,9 +1155,21 @@
           <t>Jiridiksyon</t>
         </is>
       </c>
-      <c r="G19" s="6" t="inlineStr"/>
-      <c r="H19" s="6" t="inlineStr"/>
-      <c r="I19" s="6" t="inlineStr"/>
+      <c r="G19" s="6" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="H19" s="6" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="I19" s="6" t="inlineStr">
+        <is>
+          <t>Confirmé par Me Vaval le 18 oct. (« auto confirm »)</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="5" t="n">
@@ -1040,9 +1200,21 @@
           <t>Tout jiridiksyon yo</t>
         </is>
       </c>
-      <c r="G20" s="6" t="inlineStr"/>
-      <c r="H20" s="6" t="inlineStr"/>
-      <c r="I20" s="6" t="inlineStr"/>
+      <c r="G20" s="6" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="H20" s="6" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="I20" s="6" t="inlineStr">
+        <is>
+          <t>Confirmé par Me Vaval le 18 oct. (« auto confirm »)</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="5" t="n">
@@ -1073,9 +1245,21 @@
           <t>{n} filt aktif</t>
         </is>
       </c>
-      <c r="G21" s="6" t="inlineStr"/>
-      <c r="H21" s="6" t="inlineStr"/>
-      <c r="I21" s="6" t="inlineStr"/>
+      <c r="G21" s="6" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="H21" s="6" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="I21" s="6" t="inlineStr">
+        <is>
+          <t>Confirmé par Me Vaval le 18 oct. (« auto confirm »)</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="5" t="n">
@@ -1106,9 +1290,21 @@
           <t>{n} filt aktif</t>
         </is>
       </c>
-      <c r="G22" s="6" t="inlineStr"/>
-      <c r="H22" s="6" t="inlineStr"/>
-      <c r="I22" s="6" t="inlineStr"/>
+      <c r="G22" s="6" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="H22" s="6" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="I22" s="6" t="inlineStr">
+        <is>
+          <t>Confirmé par Me Vaval le 18 oct. (« auto confirm »)</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="5" t="n">
@@ -1139,9 +1335,21 @@
           <t>Efase filt yo</t>
         </is>
       </c>
-      <c r="G23" s="6" t="inlineStr"/>
-      <c r="H23" s="6" t="inlineStr"/>
-      <c r="I23" s="6" t="inlineStr"/>
+      <c r="G23" s="6" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="H23" s="6" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="I23" s="6" t="inlineStr">
+        <is>
+          <t>Confirmé par Me Vaval le 18 oct. (« auto confirm »)</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="5" t="n">
@@ -1172,9 +1380,21 @@
           <t>Rechèch : « {q} »</t>
         </is>
       </c>
-      <c r="G24" s="6" t="inlineStr"/>
-      <c r="H24" s="6" t="inlineStr"/>
-      <c r="I24" s="6" t="inlineStr"/>
+      <c r="G24" s="6" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="H24" s="6" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="I24" s="6" t="inlineStr">
+        <is>
+          <t>Confirmé par Me Vaval le 18 oct. (« auto confirm »)</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="5" t="n">
@@ -1205,9 +1425,21 @@
           <t>Jiridiksyon : {name}</t>
         </is>
       </c>
-      <c r="G25" s="6" t="inlineStr"/>
-      <c r="H25" s="6" t="inlineStr"/>
-      <c r="I25" s="6" t="inlineStr"/>
+      <c r="G25" s="6" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="H25" s="6" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="I25" s="6" t="inlineStr">
+        <is>
+          <t>Confirmé par Me Vaval le 18 oct. (« auto confirm »)</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="5" t="n">
@@ -1238,9 +1470,21 @@
           <t>Komin : {name}</t>
         </is>
       </c>
-      <c r="G26" s="6" t="inlineStr"/>
-      <c r="H26" s="6" t="inlineStr"/>
-      <c r="I26" s="6" t="inlineStr"/>
+      <c r="G26" s="6" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="H26" s="6" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="I26" s="6" t="inlineStr">
+        <is>
+          <t>Confirmé par Me Vaval le 18 oct. (« auto confirm »)</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="5" t="n">
@@ -1271,9 +1515,21 @@
           <t>Retire filt la</t>
         </is>
       </c>
-      <c r="G27" s="6" t="inlineStr"/>
-      <c r="H27" s="6" t="inlineStr"/>
-      <c r="I27" s="6" t="inlineStr"/>
+      <c r="G27" s="6" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="H27" s="6" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="I27" s="6" t="inlineStr">
+        <is>
+          <t>Confirmé par Me Vaval le 18 oct. (« auto confirm »)</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="5" t="n">
@@ -1304,9 +1560,21 @@
           <t>Gade tout notè yo</t>
         </is>
       </c>
-      <c r="G28" s="6" t="inlineStr"/>
-      <c r="H28" s="6" t="inlineStr"/>
-      <c r="I28" s="6" t="inlineStr"/>
+      <c r="G28" s="6" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="H28" s="6" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="I28" s="6" t="inlineStr">
+        <is>
+          <t>Confirmé par Me Vaval le 18 oct. (« auto confirm »)</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="5" t="n">
@@ -1337,9 +1605,21 @@
           <t>Montre kat la</t>
         </is>
       </c>
-      <c r="G29" s="6" t="inlineStr"/>
-      <c r="H29" s="6" t="inlineStr"/>
-      <c r="I29" s="6" t="inlineStr"/>
+      <c r="G29" s="6" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="H29" s="6" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="I29" s="6" t="inlineStr">
+        <is>
+          <t>Confirmé par Me Vaval le 18 oct. (« auto confirm »)</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="5" t="n">
@@ -1370,9 +1650,21 @@
           <t>Kache kat la</t>
         </is>
       </c>
-      <c r="G30" s="6" t="inlineStr"/>
-      <c r="H30" s="6" t="inlineStr"/>
-      <c r="I30" s="6" t="inlineStr"/>
+      <c r="G30" s="6" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="H30" s="6" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="I30" s="6" t="inlineStr">
+        <is>
+          <t>Confirmé par Me Vaval le 18 oct. (« auto confirm »)</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="5" t="n">
@@ -1403,9 +1695,21 @@
           <t>Kat notè yo pa komin</t>
         </is>
       </c>
-      <c r="G31" s="6" t="inlineStr"/>
-      <c r="H31" s="6" t="inlineStr"/>
-      <c r="I31" s="6" t="inlineStr"/>
+      <c r="G31" s="6" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="H31" s="6" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="I31" s="6" t="inlineStr">
+        <is>
+          <t>Confirmé par Me Vaval le 18 oct. (« auto confirm »)</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="5" t="n">
@@ -1436,9 +1740,21 @@
           <t>Sou kat la, chak notè parèt nan komin komisyon li : kote etid yo ye a pa jewolokalize.</t>
         </is>
       </c>
-      <c r="G32" s="6" t="inlineStr"/>
-      <c r="H32" s="6" t="inlineStr"/>
-      <c r="I32" s="6" t="inlineStr"/>
+      <c r="G32" s="6" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="H32" s="6" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="I32" s="6" t="inlineStr">
+        <is>
+          <t>Confirmé par Me Vaval le 18 oct. (« auto confirm »)</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="5" t="n">
@@ -1469,9 +1785,21 @@
           <t>Rezilta anyè a</t>
         </is>
       </c>
-      <c r="G33" s="6" t="inlineStr"/>
-      <c r="H33" s="6" t="inlineStr"/>
-      <c r="I33" s="6" t="inlineStr"/>
+      <c r="G33" s="6" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="H33" s="6" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="I33" s="6" t="inlineStr">
+        <is>
+          <t>Confirmé par Me Vaval le 18 oct. (« auto confirm »)</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="5" t="n">
@@ -1502,9 +1830,21 @@
           <t>{n} notè</t>
         </is>
       </c>
-      <c r="G34" s="6" t="inlineStr"/>
-      <c r="H34" s="6" t="inlineStr"/>
-      <c r="I34" s="6" t="inlineStr"/>
+      <c r="G34" s="6" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="H34" s="6" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="I34" s="6" t="inlineStr">
+        <is>
+          <t>Confirmé par Me Vaval le 18 oct. (« auto confirm »)</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="5" t="n">
@@ -1535,9 +1875,21 @@
           <t>{n} notè</t>
         </is>
       </c>
-      <c r="G35" s="6" t="inlineStr"/>
-      <c r="H35" s="6" t="inlineStr"/>
-      <c r="I35" s="6" t="inlineStr"/>
+      <c r="G35" s="6" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="H35" s="6" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="I35" s="6" t="inlineStr">
+        <is>
+          <t>Confirmé par Me Vaval le 18 oct. (« auto confirm »)</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="5" t="n">
@@ -1568,9 +1920,21 @@
           <t>{from}–{to} sou {n}</t>
         </is>
       </c>
-      <c r="G36" s="6" t="inlineStr"/>
-      <c r="H36" s="6" t="inlineStr"/>
-      <c r="I36" s="6" t="inlineStr"/>
+      <c r="G36" s="6" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="H36" s="6" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="I36" s="6" t="inlineStr">
+        <is>
+          <t>Confirmé par Me Vaval le 18 oct. (« auto confirm »)</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="5" t="n">
@@ -1601,9 +1965,21 @@
           <t>N ap mete lis la ajou…</t>
         </is>
       </c>
-      <c r="G37" s="6" t="inlineStr"/>
-      <c r="H37" s="6" t="inlineStr"/>
-      <c r="I37" s="6" t="inlineStr"/>
+      <c r="G37" s="6" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="H37" s="6" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="I37" s="6" t="inlineStr">
+        <is>
+          <t>Confirmé par Me Vaval le 18 oct. (« auto confirm »)</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="5" t="n">
@@ -1634,9 +2010,21 @@
           <t>Pa gen notè ki koresponn ak kritè sa yo.</t>
         </is>
       </c>
-      <c r="G38" s="6" t="inlineStr"/>
-      <c r="H38" s="6" t="inlineStr"/>
-      <c r="I38" s="6" t="inlineStr"/>
+      <c r="G38" s="6" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="H38" s="6" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="I38" s="6" t="inlineStr">
+        <is>
+          <t>Confirmé par Me Vaval le 18 oct. (« auto confirm »)</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="5" t="n">
@@ -1667,9 +2055,21 @@
           <t>Chanje rechèch la oswa efase filt yo.</t>
         </is>
       </c>
-      <c r="G39" s="6" t="inlineStr"/>
-      <c r="H39" s="6" t="inlineStr"/>
-      <c r="I39" s="6" t="inlineStr"/>
+      <c r="G39" s="6" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="H39" s="6" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="I39" s="6" t="inlineStr">
+        <is>
+          <t>Confirmé par Me Vaval le 18 oct. (« auto confirm »)</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="5" t="n">
@@ -1700,9 +2100,21 @@
           <t>Anyè a pa t ka chaje.</t>
         </is>
       </c>
-      <c r="G40" s="6" t="inlineStr"/>
-      <c r="H40" s="6" t="inlineStr"/>
-      <c r="I40" s="6" t="inlineStr"/>
+      <c r="G40" s="6" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="H40" s="6" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="I40" s="6" t="inlineStr">
+        <is>
+          <t>Confirmé par Me Vaval le 18 oct. (« auto confirm »)</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="5" t="n">
@@ -1733,9 +2145,21 @@
           <t>Yon pwoblèm anpeche nou montre notè yo kounye a : lis la pa vid. Eseye ankò nan yon ti moman.</t>
         </is>
       </c>
-      <c r="G41" s="6" t="inlineStr"/>
-      <c r="H41" s="6" t="inlineStr"/>
-      <c r="I41" s="6" t="inlineStr"/>
+      <c r="G41" s="6" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="H41" s="6" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="I41" s="6" t="inlineStr">
+        <is>
+          <t>Confirmé par Me Vaval le 18 oct. (« auto confirm »)</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="5" t="n">
@@ -1766,9 +2190,21 @@
           <t>Eseye ankò</t>
         </is>
       </c>
-      <c r="G42" s="6" t="inlineStr"/>
-      <c r="H42" s="6" t="inlineStr"/>
-      <c r="I42" s="6" t="inlineStr"/>
+      <c r="G42" s="6" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="H42" s="6" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="I42" s="6" t="inlineStr">
+        <is>
+          <t>Confirmé par Me Vaval le 18 oct. (« auto confirm »)</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="5" t="n">
@@ -1799,9 +2235,21 @@
           <t>Komin komisyon</t>
         </is>
       </c>
-      <c r="G43" s="6" t="inlineStr"/>
-      <c r="H43" s="6" t="inlineStr"/>
-      <c r="I43" s="6" t="inlineStr"/>
+      <c r="G43" s="6" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="H43" s="6" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="I43" s="6" t="inlineStr">
+        <is>
+          <t>Confirmé par Me Vaval le 18 oct. (« auto confirm »)</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="5" t="n">
@@ -1832,9 +2280,21 @@
           <t>Adrès etid la</t>
         </is>
       </c>
-      <c r="G44" s="6" t="inlineStr"/>
-      <c r="H44" s="6" t="inlineStr"/>
-      <c r="I44" s="6" t="inlineStr"/>
+      <c r="G44" s="6" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="H44" s="6" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="I44" s="6" t="inlineStr">
+        <is>
+          <t>Confirmé par Me Vaval le 18 oct. (« auto confirm »)</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="5" t="n">
@@ -1865,7 +2325,11 @@
           <t>Adrès etid la pa kominike</t>
         </is>
       </c>
-      <c r="G45" s="6" t="n"/>
+      <c r="G45" s="6" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
       <c r="H45" s="6" t="inlineStr">
         <is>
           <t>Oui</t>
@@ -1906,9 +2370,21 @@
           <t>{address} — gade komin {commune} sou kat la (etid la pa jewolokalize)</t>
         </is>
       </c>
-      <c r="G46" s="6" t="inlineStr"/>
-      <c r="H46" s="6" t="inlineStr"/>
-      <c r="I46" s="6" t="inlineStr"/>
+      <c r="G46" s="6" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="H46" s="6" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="I46" s="6" t="inlineStr">
+        <is>
+          <t>Confirmé par Me Vaval le 18 oct. (« auto confirm »)</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="5" t="n">
@@ -1939,9 +2415,21 @@
           <t>Montre komin nan sou kat la</t>
         </is>
       </c>
-      <c r="G47" s="6" t="inlineStr"/>
-      <c r="H47" s="6" t="inlineStr"/>
-      <c r="I47" s="6" t="inlineStr"/>
+      <c r="G47" s="6" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="H47" s="6" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="I47" s="6" t="inlineStr">
+        <is>
+          <t>Confirmé par Me Vaval le 18 oct. (« auto confirm »)</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="5" t="n">
@@ -1972,9 +2460,21 @@
           <t>Montre sou kat la komin {commune}, kote {name} komisyone</t>
         </is>
       </c>
-      <c r="G48" s="6" t="inlineStr"/>
-      <c r="H48" s="6" t="inlineStr"/>
-      <c r="I48" s="6" t="inlineStr"/>
+      <c r="G48" s="6" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="H48" s="6" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="I48" s="6" t="inlineStr">
+        <is>
+          <t>Confirmé par Me Vaval le 18 oct. (« auto confirm »)</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="5" t="n">
@@ -2005,9 +2505,21 @@
           <t>Gade fich la</t>
         </is>
       </c>
-      <c r="G49" s="6" t="inlineStr"/>
-      <c r="H49" s="6" t="inlineStr"/>
-      <c r="I49" s="6" t="inlineStr"/>
+      <c r="G49" s="6" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="H49" s="6" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="I49" s="6" t="inlineStr">
+        <is>
+          <t>Confirmé par Me Vaval le 18 oct. (« auto confirm »)</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="5" t="n">
@@ -2038,9 +2550,21 @@
           <t>Gade fich {name}</t>
         </is>
       </c>
-      <c r="G50" s="6" t="inlineStr"/>
-      <c r="H50" s="6" t="inlineStr"/>
-      <c r="I50" s="6" t="inlineStr"/>
+      <c r="G50" s="6" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="H50" s="6" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="I50" s="6" t="inlineStr">
+        <is>
+          <t>Confirmé par Me Vaval le 18 oct. (« auto confirm »)</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="5" t="n">
@@ -2071,9 +2595,21 @@
           <t>kontinyasyon</t>
         </is>
       </c>
-      <c r="G51" s="6" t="inlineStr"/>
-      <c r="H51" s="6" t="inlineStr"/>
-      <c r="I51" s="6" t="inlineStr"/>
+      <c r="G51" s="6" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="H51" s="6" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="I51" s="6" t="inlineStr">
+        <is>
+          <t>Confirmé par Me Vaval le 18 oct. (« auto confirm »)</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="5" t="n">
@@ -2104,9 +2640,21 @@
           <t>Jiridiksyon pa detèmine</t>
         </is>
       </c>
-      <c r="G52" s="6" t="inlineStr"/>
-      <c r="H52" s="6" t="inlineStr"/>
-      <c r="I52" s="6" t="inlineStr"/>
+      <c r="G52" s="6" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="H52" s="6" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="I52" s="6" t="inlineStr">
+        <is>
+          <t>Confirmé par Me Vaval le 18 oct. (« auto confirm »)</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="5" t="n">
@@ -2137,9 +2685,21 @@
           <t>komin ki enprime : {name}</t>
         </is>
       </c>
-      <c r="G53" s="6" t="inlineStr"/>
-      <c r="H53" s="6" t="inlineStr"/>
-      <c r="I53" s="6" t="inlineStr"/>
+      <c r="G53" s="6" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="H53" s="6" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="I53" s="6" t="inlineStr">
+        <is>
+          <t>Confirmé par Me Vaval le 18 oct. (« auto confirm »)</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="5" t="n">
@@ -2170,9 +2730,21 @@
           <t>Paj anyè a</t>
         </is>
       </c>
-      <c r="G54" s="6" t="inlineStr"/>
-      <c r="H54" s="6" t="inlineStr"/>
-      <c r="I54" s="6" t="inlineStr"/>
+      <c r="G54" s="6" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="H54" s="6" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="I54" s="6" t="inlineStr">
+        <is>
+          <t>Confirmé par Me Vaval le 18 oct. (« auto confirm »)</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="5" t="n">
@@ -2203,9 +2775,21 @@
           <t>Anvan</t>
         </is>
       </c>
-      <c r="G55" s="6" t="inlineStr"/>
-      <c r="H55" s="6" t="inlineStr"/>
-      <c r="I55" s="6" t="inlineStr"/>
+      <c r="G55" s="6" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="H55" s="6" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="I55" s="6" t="inlineStr">
+        <is>
+          <t>Confirmé par Me Vaval le 18 oct. (« auto confirm »)</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="5" t="n">
@@ -2236,9 +2820,21 @@
           <t>Apre</t>
         </is>
       </c>
-      <c r="G56" s="6" t="inlineStr"/>
-      <c r="H56" s="6" t="inlineStr"/>
-      <c r="I56" s="6" t="inlineStr"/>
+      <c r="G56" s="6" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="H56" s="6" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="I56" s="6" t="inlineStr">
+        <is>
+          <t>Confirmé par Me Vaval le 18 oct. (« auto confirm »)</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="5" t="n">
@@ -2269,9 +2865,21 @@
           <t>Paj {n}</t>
         </is>
       </c>
-      <c r="G57" s="6" t="inlineStr"/>
-      <c r="H57" s="6" t="inlineStr"/>
-      <c r="I57" s="6" t="inlineStr"/>
+      <c r="G57" s="6" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="H57" s="6" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="I57" s="6" t="inlineStr">
+        <is>
+          <t>Confirmé par Me Vaval le 18 oct. (« auto confirm »)</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="5" t="n">
@@ -2302,9 +2910,21 @@
           <t>Anyè a repwodui lis MJSP pibliye a ; nou pa prezante l kòm konplè. Adrès etid yo te kominike bay redaksyon Agora.</t>
         </is>
       </c>
-      <c r="G58" s="6" t="inlineStr"/>
-      <c r="H58" s="6" t="inlineStr"/>
-      <c r="I58" s="6" t="inlineStr"/>
+      <c r="G58" s="6" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="H58" s="6" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="I58" s="6" t="inlineStr">
+        <is>
+          <t>Confirmé par Me Vaval le 18 oct. (« auto confirm »)</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="5" t="n">
@@ -2335,9 +2955,21 @@
           <t>Klasman : pa jiridiksyon, etid ki gen adrès yo an premye, apre pa non fanmi.</t>
         </is>
       </c>
-      <c r="G59" s="6" t="inlineStr"/>
-      <c r="H59" s="6" t="inlineStr"/>
-      <c r="I59" s="6" t="inlineStr"/>
+      <c r="G59" s="6" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="H59" s="6" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="I59" s="6" t="inlineStr">
+        <is>
+          <t>Confirmé par Me Vaval le 18 oct. (« auto confirm »)</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="5" t="n">
@@ -2368,9 +3000,21 @@
           <t>Retounen nan anyè a</t>
         </is>
       </c>
-      <c r="G60" s="6" t="inlineStr"/>
-      <c r="H60" s="6" t="inlineStr"/>
-      <c r="I60" s="6" t="inlineStr"/>
+      <c r="G60" s="6" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="H60" s="6" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="I60" s="6" t="inlineStr">
+        <is>
+          <t>Confirmé par Me Vaval le 18 oct. (« auto confirm »)</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="5" t="n">
@@ -2401,9 +3045,21 @@
           <t>Notè</t>
         </is>
       </c>
-      <c r="G61" s="6" t="inlineStr"/>
-      <c r="H61" s="6" t="inlineStr"/>
-      <c r="I61" s="6" t="inlineStr"/>
+      <c r="G61" s="6" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="H61" s="6" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="I61" s="6" t="inlineStr">
+        <is>
+          <t>Confirmé par Me Vaval le 18 oct. (« auto confirm »)</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="5" t="n">
@@ -2434,9 +3090,21 @@
           <t>Konfime</t>
         </is>
       </c>
-      <c r="G62" s="6" t="inlineStr"/>
-      <c r="H62" s="6" t="inlineStr"/>
-      <c r="I62" s="6" t="inlineStr"/>
+      <c r="G62" s="6" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="H62" s="6" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="I62" s="6" t="inlineStr">
+        <is>
+          <t>Confirmé par Me Vaval le 18 oct. (« auto confirm »)</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="5" t="n">
@@ -2467,7 +3135,11 @@
           <t>Notè a konfime enfòmasyon an.</t>
         </is>
       </c>
-      <c r="G63" s="6" t="n"/>
+      <c r="G63" s="6" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
       <c r="H63" s="6" t="inlineStr">
         <is>
           <t>Oui</t>
@@ -2508,11 +3180,19 @@
           <t>Notè a konfime enfòmasyon an</t>
         </is>
       </c>
-      <c r="G64" s="6" t="inlineStr"/>
-      <c r="H64" s="6" t="inlineStr"/>
+      <c r="G64" s="6" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="H64" s="6" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
       <c r="I64" s="6" t="inlineStr">
         <is>
-          <t>Aligné sur sa correction de l’infobulle — à valider</t>
+          <t>Aligné sur sa correction de l’infobulle — confirmé (« auto confirm »)</t>
         </is>
       </c>
     </row>
@@ -2545,9 +3225,21 @@
           <t>Konfime {date}</t>
         </is>
       </c>
-      <c r="G65" s="6" t="inlineStr"/>
-      <c r="H65" s="6" t="inlineStr"/>
-      <c r="I65" s="6" t="inlineStr"/>
+      <c r="G65" s="6" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="H65" s="6" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="I65" s="6" t="inlineStr">
+        <is>
+          <t>Confirmé par Me Vaval le 18 oct. (« auto confirm »)</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="5" t="n">
@@ -2578,9 +3270,21 @@
           <t>Mande yon koreksyon oswa yon konfimasyon</t>
         </is>
       </c>
-      <c r="G66" s="6" t="inlineStr"/>
-      <c r="H66" s="6" t="inlineStr"/>
-      <c r="I66" s="6" t="inlineStr"/>
+      <c r="G66" s="6" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="H66" s="6" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="I66" s="6" t="inlineStr">
+        <is>
+          <t>Confirmé par Me Vaval le 18 oct. (« auto confirm »)</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="5" t="n">
@@ -2611,11 +3315,19 @@
           <t>Pwopoze yon koreksyon oswa konfime enfòmasyon ki afiche yo. Administratè a ap egzamine demann lan : anyen p ap pibliye anvan verifikasyon.</t>
         </is>
       </c>
-      <c r="G67" s="6" t="inlineStr"/>
-      <c r="H67" s="6" t="inlineStr"/>
+      <c r="G67" s="6" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="H67" s="6" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
       <c r="I67" s="6" t="inlineStr">
         <is>
-          <t>Aligné sur « l’Administrateur » (sa correction du message d’envoi) — à valider</t>
+          <t>Aligné sur « l’Administrateur » (sa correction du message d’envoi) — confirmé (« auto confirm »)</t>
         </is>
       </c>
     </row>
@@ -2648,9 +3360,21 @@
           <t>Youn oswa plizyè imel, separe ak yon pwen-vigil.</t>
         </is>
       </c>
-      <c r="G68" s="6" t="inlineStr"/>
-      <c r="H68" s="6" t="inlineStr"/>
-      <c r="I68" s="6" t="inlineStr"/>
+      <c r="G68" s="6" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="H68" s="6" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="I68" s="6" t="inlineStr">
+        <is>
+          <t>Confirmé par Me Vaval le 18 oct. (« auto confirm »)</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="5" t="n">
@@ -2726,9 +3450,21 @@
           <t>Mande yon koreksyon</t>
         </is>
       </c>
-      <c r="G70" s="6" t="inlineStr"/>
-      <c r="H70" s="6" t="inlineStr"/>
-      <c r="I70" s="6" t="inlineStr"/>
+      <c r="G70" s="6" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="H70" s="6" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="I70" s="6" t="inlineStr">
+        <is>
+          <t>Confirmé par Me Vaval le 18 oct. (« auto confirm »)</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="5" t="n">
@@ -2759,9 +3495,21 @@
           <t>Konfime enfòmasyon ki afiche yo</t>
         </is>
       </c>
-      <c r="G71" s="6" t="inlineStr"/>
-      <c r="H71" s="6" t="inlineStr"/>
-      <c r="I71" s="6" t="inlineStr"/>
+      <c r="G71" s="6" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="H71" s="6" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="I71" s="6" t="inlineStr">
+        <is>
+          <t>Confirmé par Me Vaval le 18 oct. (« auto confirm »)</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="5" t="n">
@@ -2792,9 +3540,21 @@
           <t>Chan yo reprann enfòmasyon ki pibliye yo : chanje sa ki pou korije yo.</t>
         </is>
       </c>
-      <c r="G72" s="6" t="inlineStr"/>
-      <c r="H72" s="6" t="inlineStr"/>
-      <c r="I72" s="6" t="inlineStr"/>
+      <c r="G72" s="6" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="H72" s="6" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="I72" s="6" t="inlineStr">
+        <is>
+          <t>Confirmé par Me Vaval le 18 oct. (« auto confirm »)</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="5" t="n">
@@ -2825,9 +3585,21 @@
           <t>Men enfòmasyon ki pibliye sou fich la. Si yo egzat, konfime yo : redaksyon an ap verifye kote demann lan soti anvan badj « Konfime » parèt.</t>
         </is>
       </c>
-      <c r="G73" s="6" t="inlineStr"/>
-      <c r="H73" s="6" t="inlineStr"/>
-      <c r="I73" s="6" t="inlineStr"/>
+      <c r="G73" s="6" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="H73" s="6" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="I73" s="6" t="inlineStr">
+        <is>
+          <t>Confirmé par Me Vaval le 18 oct. (« auto confirm »)</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="5" t="n">
@@ -2858,9 +3630,21 @@
           <t>Enfòmasyon ki pibliye</t>
         </is>
       </c>
-      <c r="G74" s="6" t="inlineStr"/>
-      <c r="H74" s="6" t="inlineStr"/>
-      <c r="I74" s="6" t="inlineStr"/>
+      <c r="G74" s="6" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="H74" s="6" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="I74" s="6" t="inlineStr">
+        <is>
+          <t>Confirmé par Me Vaval le 18 oct. (« auto confirm »)</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="5" t="n">
@@ -2891,9 +3675,21 @@
           <t>Mwen konfime enfòmasyon ki afiche yo egzat.</t>
         </is>
       </c>
-      <c r="G75" s="6" t="inlineStr"/>
-      <c r="H75" s="6" t="inlineStr"/>
-      <c r="I75" s="6" t="inlineStr"/>
+      <c r="G75" s="6" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="H75" s="6" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="I75" s="6" t="inlineStr">
+        <is>
+          <t>Confirmé par Me Vaval le 18 oct. (« auto confirm »)</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="5" t="n">
@@ -2924,11 +3720,19 @@
           <t>pa kominike</t>
         </is>
       </c>
-      <c r="G76" s="6" t="inlineStr"/>
-      <c r="H76" s="6" t="inlineStr"/>
+      <c r="G76" s="6" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="H76" s="6" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
       <c r="I76" s="6" t="inlineStr">
         <is>
-          <t>Aligné sur « pa kominike » — à valider</t>
+          <t>Aligné sur « pa kominike » — confirmé (« auto confirm »)</t>
         </is>
       </c>
     </row>
@@ -2961,9 +3765,21 @@
           <t>tcheke ti kare konfimasyon an</t>
         </is>
       </c>
-      <c r="G77" s="6" t="inlineStr"/>
-      <c r="H77" s="6" t="inlineStr"/>
-      <c r="I77" s="6" t="inlineStr"/>
+      <c r="G77" s="6" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="H77" s="6" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="I77" s="6" t="inlineStr">
+        <is>
+          <t>Confirmé par Me Vaval le 18 oct. (« auto confirm »)</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="5" t="n">
@@ -2994,9 +3810,21 @@
           <t>enfòmasyon fich la chanje depi fòmilè a te parèt ; rechaje paj la epi verifye yo ankò</t>
         </is>
       </c>
-      <c r="G78" s="6" t="inlineStr"/>
-      <c r="H78" s="6" t="inlineStr"/>
-      <c r="I78" s="6" t="inlineStr"/>
+      <c r="G78" s="6" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="H78" s="6" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="I78" s="6" t="inlineStr">
+        <is>
+          <t>Confirmé par Me Vaval le 18 oct. (« auto confirm »)</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="5" t="n">
@@ -3027,9 +3855,21 @@
           <t>Demann lan voye</t>
         </is>
       </c>
-      <c r="G79" s="6" t="inlineStr"/>
-      <c r="H79" s="6" t="inlineStr"/>
-      <c r="I79" s="6" t="inlineStr"/>
+      <c r="G79" s="6" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="H79" s="6" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="I79" s="6" t="inlineStr">
+        <is>
+          <t>Confirmé par Me Vaval le 18 oct. (« auto confirm »)</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <dataValidations count="1">

</xml_diff>